<commit_message>
- Update CoreCollectedDataDeletionUtil to delete XML and media files using just CoreCollectedData - its easier and faster - Fix constructor calls for RegionFormUtil, HouseholdFormUtil and PreHouseholdFormUtil - Fix missing SyncReport with entity SyncEntity.CORE_FORMS_OPTIONS on Bootstrap - Fix missing filename on SyncEntitiesTask.downloadCoreFormExtensionsFiles - Fix missing Loading Dialog when opening Extension Forms
</commit_message>
<xml_diff>
--- a/app/src/main/res/raw/household_form.xlsx
+++ b/app/src/main/res/raw/household_form.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27795" windowHeight="12195" tabRatio="500"/>
+    <workbookView windowWidth="27795" windowHeight="12315" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="columns" sheetId="1" r:id="rId1"/>
@@ -15,8 +15,42 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>paul</author>
+  </authors>
+  <commentList>
+    <comment ref="G1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="134"/>
+          </rPr>
+          <t>paul:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <rFont val="Times New Roman"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+The option is readonly, not choosable.
+Only selectable programatically, when selected make the all options read-only
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="208">
   <si>
     <t>group</t>
   </si>
@@ -51,6 +85,12 @@
     <t>label::am</t>
   </si>
   <si>
+    <t>validation</t>
+  </si>
+  <si>
+    <t>validation_message</t>
+  </si>
+  <si>
     <t>default_value</t>
   </si>
   <si>
@@ -610,6 +650,15 @@
   </si>
   <si>
     <t>form_name::am</t>
+  </si>
+  <si>
+    <t>form_version</t>
+  </si>
+  <si>
+    <t>repeat_name</t>
+  </si>
+  <si>
+    <t>repeat_xml_node</t>
   </si>
   <si>
     <t>rawHousehold</t>
@@ -632,12 +681,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="179" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -645,9 +694,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -676,14 +731,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -699,14 +746,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
@@ -714,10 +753,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color theme="3"/>
       <name val="Arial"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -729,15 +769,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FF800080"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -745,7 +787,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -766,6 +808,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
@@ -775,7 +831,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFA7D00"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -783,17 +839,21 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Arial"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Arial"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="34">
@@ -811,37 +871,133 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -853,49 +1009,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -907,7 +1027,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -919,84 +1051,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="16">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -1082,11 +1142,63 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1108,24 +1220,20 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1144,200 +1252,165 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1354,19 +1427,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -1683,7 +1756,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R30"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="12.75"/>
   <cols>
     <col min="2" max="2" width="11.1809523809524" customWidth="1"/>
@@ -1695,15 +1768,16 @@
     <col min="8" max="8" width="39.6" customWidth="1"/>
     <col min="9" max="9" width="41.2761904761905" customWidth="1"/>
     <col min="10" max="10" width="40.5714285714286" customWidth="1"/>
-    <col min="11" max="11" width="34.5714285714286" customWidth="1"/>
-    <col min="12" max="12" width="21.7238095238095" customWidth="1"/>
-    <col min="13" max="13" width="10.4571428571429" customWidth="1"/>
-    <col min="14" max="14" width="9.26666666666667" customWidth="1"/>
-    <col min="16" max="16" width="36" customWidth="1"/>
-    <col min="17" max="17" width="12.7142857142857" customWidth="1"/>
+    <col min="11" max="12" width="34.5714285714286" customWidth="1"/>
+    <col min="13" max="13" width="42.7619047619048" customWidth="1"/>
+    <col min="14" max="14" width="21.7238095238095" customWidth="1"/>
+    <col min="15" max="15" width="10.4571428571429" customWidth="1"/>
+    <col min="16" max="16" width="9.26666666666667" customWidth="1"/>
+    <col min="18" max="18" width="36" customWidth="1"/>
+    <col min="19" max="19" width="12.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1749,443 +1823,483 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="19" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="I2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" t="b">
+      <c r="H3" t="s">
+        <v>29</v>
+      </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="Q3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="I3" t="s">
-        <v>28</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" t="b">
+      <c r="D4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" t="b">
         <v>1</v>
       </c>
-      <c r="O3" t="b">
+      <c r="Q4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" t="b">
-        <v>1</v>
-      </c>
-      <c r="O4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:16">
       <c r="A5" s="1"/>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>40</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="K5" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="L5" s="13"/>
-      <c r="M5" s="13"/>
-      <c r="N5" t="b">
+      <c r="J5" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="K5" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="L5" s="14"/>
+      <c r="M5" s="14"/>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14"/>
+      <c r="P5" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:18">
       <c r="A6" s="1"/>
       <c r="D6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I6" t="s">
-        <v>46</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="K6" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" t="b">
+      <c r="J6" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" s="14"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" t="b">
         <v>1</v>
       </c>
-      <c r="P6" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16">
+      <c r="R6" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:18">
       <c r="A7" s="1"/>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>52</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K7" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" t="b">
+      <c r="J7" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="14"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" t="b">
         <v>1</v>
       </c>
-      <c r="P7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14">
+      <c r="R7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
       <c r="A8" s="1"/>
       <c r="D8" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K8" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" t="b">
+      <c r="J8" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="14"/>
+      <c r="M8" s="14"/>
+      <c r="N8" s="14"/>
+      <c r="O8" s="14"/>
+      <c r="P8" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:17">
       <c r="A9" s="1"/>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="I9" t="s">
-        <v>63</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="K9" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="O9" t="b">
+      <c r="J9" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="K9" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="L9" s="14"/>
+      <c r="M9" s="14"/>
+      <c r="N9" s="14"/>
+      <c r="O9" s="14"/>
+      <c r="Q9" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:17">
       <c r="A10" s="1"/>
       <c r="D10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>68</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="K10" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="L10" s="13"/>
-      <c r="M10" s="13"/>
-      <c r="O10" t="b">
+      <c r="J10" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="K10" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="Q10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:16">
       <c r="A11" s="1"/>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I11" t="s">
-        <v>73</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="K11" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="20"/>
-    </row>
-    <row r="12" s="5" customFormat="1" ht="13" customHeight="1" spans="1:15">
+      <c r="J11" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="K11" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="22"/>
+    </row>
+    <row r="12" s="5" customFormat="1" ht="13" customHeight="1" spans="1:17">
       <c r="A12" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
       <c r="H12" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="K12" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="5" t="b">
+      <c r="J12" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="L12" s="18"/>
+      <c r="M12" s="18"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="O12" s="5" t="b">
+      <c r="Q12" s="5" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" s="6" customFormat="1" spans="1:15">
+    <row r="13" s="6" customFormat="1" spans="1:17">
       <c r="A13" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="K13" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="6" t="b">
+      <c r="J13" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="K13" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="O13" s="6" t="b">
+      <c r="Q13" s="6" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" s="6" customFormat="1" spans="1:18">
+    <row r="14" s="6" customFormat="1" spans="1:20">
       <c r="A14" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="K14" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="O14" s="6" t="b">
+        <v>93</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="K14" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="Q14" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="R14" s="6" t="b">
+      <c r="T14" s="6" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" s="7" customFormat="1" spans="1:15">
+    <row r="15" s="7" customFormat="1" spans="1:17">
       <c r="A15" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E15" s="7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="K15" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
-      <c r="N15" s="7" t="b">
+      <c r="J15" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K15" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="L15" s="20"/>
+      <c r="M15" s="20"/>
+      <c r="N15" s="20"/>
+      <c r="O15" s="20"/>
+      <c r="P15" s="7" t="b">
         <v>1</v>
       </c>
-      <c r="O15" s="7" t="b">
+      <c r="Q15" s="7" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:15">
       <c r="A16" s="1"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-    </row>
-    <row r="17" spans="1:13">
+      <c r="K16" s="14"/>
+      <c r="L16" s="14"/>
+      <c r="M16" s="14"/>
+      <c r="N16" s="14"/>
+      <c r="O16" s="14"/>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" s="1"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="13"/>
-    </row>
-    <row r="18" spans="1:13">
+      <c r="K17" s="14"/>
+      <c r="L17" s="14"/>
+      <c r="M17" s="14"/>
+      <c r="N17" s="14"/>
+      <c r="O17" s="14"/>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" s="1"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="21"/>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="1"/>
@@ -2233,23 +2347,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="9.18095238095238" defaultRowHeight="12.75" outlineLevelCol="5"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultColWidth="9.18095238095238" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="15.7142857142857" customWidth="1"/>
     <col min="2" max="2" width="16.2857142857143" customWidth="1"/>
     <col min="3" max="3" width="52.4285714285714" customWidth="1"/>
-    <col min="4" max="4" width="50.0380952380952" customWidth="1"/>
-    <col min="5" max="5" width="48.4857142857143" customWidth="1"/>
-    <col min="6" max="6" width="29.8666666666667" customWidth="1"/>
+    <col min="4" max="4" width="55.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="54.1428571428571" customWidth="1"/>
+    <col min="6" max="6" width="62.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="12.3238095238095" customWidth="1"/>
+    <col min="8" max="8" width="20.8857142857143" customWidth="1"/>
+    <col min="9" max="9" width="16.247619047619" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C1" t="s">
         <v>7</v>
@@ -2263,385 +2380,460 @@
       <c r="F1" t="s">
         <v>10</v>
       </c>
+      <c r="G1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="3" t="s">
-        <v>38</v>
+      <c r="A2" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
-        <v>38</v>
+      <c r="A3" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
-        <v>44</v>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F4" t="s">
-        <v>113</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
-        <v>44</v>
+      <c r="A5" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
-        <v>44</v>
+      <c r="A6" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="F6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="4" t="s">
-        <v>44</v>
+      <c r="A7" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E7" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="4" t="s">
-        <v>44</v>
+      <c r="A8" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C8" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D8" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="4" t="s">
-        <v>44</v>
+      <c r="A9" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D9" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="4" t="s">
-        <v>44</v>
+      <c r="A10" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="4" t="s">
-        <v>44</v>
+      <c r="A11" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="4" t="s">
-        <v>44</v>
+      <c r="A12" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="E12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="4" t="s">
-        <v>44</v>
+      <c r="A13" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B13" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="4" t="s">
-        <v>44</v>
+      <c r="A14" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C14" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E14" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="4" t="s">
-        <v>44</v>
+      <c r="A15" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C15" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D15" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="E15" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F15" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="4" t="s">
-        <v>44</v>
+      <c r="A16" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C16" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="4" t="s">
-        <v>44</v>
+      <c r="A17" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C17" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="E17" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F17" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="4" t="s">
-        <v>44</v>
+      <c r="A18" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B18" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C18" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D18" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E18" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F18" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="4" t="s">
-        <v>44</v>
+      <c r="A19" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B19" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D19" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="E19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="4" t="s">
-        <v>44</v>
+      <c r="A20" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C20" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D20" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E20" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F20" t="s">
-        <v>192</v>
+        <v>194</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="9.18095238095238" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="7"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="20.4571428571429" customWidth="1"/>
+    <col min="3" max="3" width="23.2666666666667" customWidth="1"/>
+    <col min="4" max="4" width="33.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="26.1142857142857" customWidth="1"/>
+    <col min="6" max="7" width="12.5714285714286" customWidth="1"/>
+    <col min="8" max="8" width="16.4285714285714" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="E2" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -2650,55 +2842,19 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="9.18095238095238" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="4"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="20.4571428571429" customWidth="1"/>
-    <col min="3" max="3" width="23.2666666666667" customWidth="1"/>
-    <col min="4" max="4" width="33.5714285714286" customWidth="1"/>
-    <col min="5" max="5" width="26.1142857142857" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="C1" t="s">
-        <v>195</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="E1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E2" t="s">
-        <v>202</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <commentList sheetStid="2">
+    <comment s:ref="G1" rgbClr="BD6480"/>
+  </commentList>
+</comments>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06A0048C-2381-489B-AA07-9611017176EA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="https://web.wps.cn/et/2018/main"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>